<commit_message>
set random seem to scenario number for consistency
</commit_message>
<xml_diff>
--- a/Two Stage Deterministic equivalent/generated_random_demand_scenarios.xlsx
+++ b/Two Stage Deterministic equivalent/generated_random_demand_scenarios.xlsx
@@ -1,43 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10513"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/Two Stage Deterministic equivalent/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felipenoris/tmp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="115_{41451D9D-F397-4D8C-8901-3539EDD56976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94663383-74EF-4642-94E3-28B8D82829EE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C353BCB8-5EC8-0143-BDD3-A1B661DAACD7}" xr6:coauthVersionLast="33" xr6:coauthVersionMax="33" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{52D9C27D-0EF6-DD41-9728-0267E68F7539}"/>
+    <workbookView xWindow="380" yWindow="460" windowWidth="28040" windowHeight="17040" xr2:uid="{52D9C27D-0EF6-DD41-9728-0267E68F7539}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenario_1" sheetId="1" r:id="rId1"/>
-    <sheet name="Scenario_2" sheetId="2" r:id="rId2"/>
+    <sheet name="Scenario_2" r:id="rId5" sheetId="2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="23">
   <si>
     <t>Vaccine</t>
   </si>
@@ -161,9 +150,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -201,7 +190,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -307,7 +296,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -449,18 +438,18 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF5B91EC-1403-4310-B069-112A91895011}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF0E20E-E4D8-9B45-9C94-E89B574F109C}">
   <dimension ref="A1:K13"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -495,424 +484,424 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
         <v>11</v>
       </c>
       <c r="B2">
-        <v>229728019.87109706</v>
+        <v>2.3142376368608567e8</v>
       </c>
       <c r="C2">
-        <v>278181430.90289623</v>
+        <v>2.692875969936613e8</v>
       </c>
       <c r="D2">
-        <v>277730591.78794605</v>
+        <v>2.487086997182661e8</v>
       </c>
       <c r="E2">
-        <v>344709977.6918065</v>
+        <v>4.310252102746217e8</v>
       </c>
       <c r="F2">
-        <v>199286852.73804203</v>
+        <v>4.3873203777158517e8</v>
       </c>
       <c r="G2">
-        <v>336387529.94491667</v>
+        <v>4.01228228645577e8</v>
       </c>
       <c r="H2">
-        <v>221668509.54371643</v>
+        <v>6.51254516408437e8</v>
       </c>
       <c r="I2">
-        <v>532545604.11893821</v>
+        <v>3.0199030442409337e8</v>
       </c>
       <c r="J2">
-        <v>701920293.08618248</v>
+        <v>2.707246016457612e8</v>
       </c>
       <c r="K2">
-        <v>619832276.83044362</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4.4933700954943514e8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3" t="s">
         <v>12</v>
       </c>
       <c r="B3">
-        <v>507259532.63244545</v>
+        <v>4.0613805639822865e8</v>
       </c>
       <c r="C3">
-        <v>301962670.46680188</v>
+        <v>6.890368415514586e8</v>
       </c>
       <c r="D3">
-        <v>282047916.52857798</v>
+        <v>6.387086342140454e8</v>
       </c>
       <c r="E3">
-        <v>977377965.22984505</v>
+        <v>5.980375859255544e8</v>
       </c>
       <c r="F3">
-        <v>874627633.58146095</v>
+        <v>1.0360559225448943e9</v>
       </c>
       <c r="G3">
-        <v>606828111.85025001</v>
+        <v>8.771550571483468e8</v>
       </c>
       <c r="H3">
-        <v>1096928965.4296257</v>
+        <v>8.630765640926757e8</v>
       </c>
       <c r="I3">
-        <v>1298632127.1908684</v>
+        <v>8.551504877310476e8</v>
       </c>
       <c r="J3">
-        <v>925450428.31077075</v>
+        <v>7.671605542869583e8</v>
       </c>
       <c r="K3">
-        <v>380743917.85509372</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1.0438743421572417e9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
       <c r="A4" t="s">
         <v>13</v>
       </c>
       <c r="B4">
-        <v>31891504.127975341</v>
+        <v>3.2381396331380807e7</v>
       </c>
       <c r="C4">
-        <v>37527250.599361941</v>
+        <v>1.814613097536783e7</v>
       </c>
       <c r="D4">
-        <v>13555404.011968404</v>
+        <v>2.6059274594171997e7</v>
       </c>
       <c r="E4">
-        <v>22984386.265572675</v>
+        <v>4.611624332416355e7</v>
       </c>
       <c r="F4">
-        <v>12842956.921020798</v>
+        <v>2.961676852362835e7</v>
       </c>
       <c r="G4">
-        <v>19583767.502586585</v>
+        <v>7.455956742057548e7</v>
       </c>
       <c r="H4">
-        <v>42841912.430671223</v>
+        <v>6.666527236443293e7</v>
       </c>
       <c r="I4">
-        <v>10954964.635472097</v>
+        <v>1.045063389444261e8</v>
       </c>
       <c r="J4">
-        <v>34959119.607848644</v>
+        <v>1.1509664714493945e7</v>
       </c>
       <c r="K4">
-        <v>58241172.413923293</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1.9015579800588712e7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
       <c r="A5" t="s">
         <v>14</v>
       </c>
       <c r="B5">
-        <v>28963052.208541505</v>
+        <v>3.0277621694231816e7</v>
       </c>
       <c r="C5">
-        <v>35827721.918152146</v>
+        <v>3.518204250557581e7</v>
       </c>
       <c r="D5">
-        <v>41632699.563409016</v>
+        <v>4.383163394280776e7</v>
       </c>
       <c r="E5">
-        <v>46754645.53507138</v>
+        <v>5.152880022963601e7</v>
       </c>
       <c r="F5">
-        <v>52251559.565770455</v>
+        <v>5.1062113137056105e7</v>
       </c>
       <c r="G5">
-        <v>61319759.672927991</v>
+        <v>6.112615549295937e7</v>
       </c>
       <c r="H5">
-        <v>66941405.664307028</v>
+        <v>6.43233673561126e7</v>
       </c>
       <c r="I5">
-        <v>85959977.64408125</v>
+        <v>7.763900492216887e7</v>
       </c>
       <c r="J5">
-        <v>76682403.409934819</v>
+        <v>8.079120731954698e7</v>
       </c>
       <c r="K5">
-        <v>84229838.337548688</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+        <v>7.212549466343203e7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
       <c r="A6" t="s">
         <v>15</v>
       </c>
       <c r="B6">
-        <v>318547489.41491944</v>
+        <v>2.8515154056163275e8</v>
       </c>
       <c r="C6">
-        <v>319586231.03825468</v>
+        <v>3.4277217916061234e8</v>
       </c>
       <c r="D6">
-        <v>317049776.13664007</v>
+        <v>2.9925309266955477e8</v>
       </c>
       <c r="E6">
-        <v>358977462.51181316</v>
+        <v>3.132680111502295e8</v>
       </c>
       <c r="F6">
-        <v>428070186.99077648</v>
+        <v>3.411721682000833e8</v>
       </c>
       <c r="G6">
-        <v>425314023.75192946</v>
+        <v>3.559836374240919e8</v>
       </c>
       <c r="H6">
-        <v>318386411.4434073</v>
+        <v>4.23806403937963e8</v>
       </c>
       <c r="I6">
-        <v>381261177.62551033</v>
+        <v>4.1378236512754774e8</v>
       </c>
       <c r="J6">
-        <v>450734042.94048089</v>
+        <v>4.2134888714824206e8</v>
       </c>
       <c r="K6">
-        <v>432953084.42980027</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3.102667132423103e8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
       <c r="A7" t="s">
         <v>16</v>
       </c>
       <c r="B7">
-        <v>357228338.46645576</v>
+        <v>3.516118821112036e8</v>
       </c>
       <c r="C7">
-        <v>332997858.55895269</v>
+        <v>3.147109485428969e8</v>
       </c>
       <c r="D7">
-        <v>285958947.10065317</v>
+        <v>3.518178282918095e8</v>
       </c>
       <c r="E7">
-        <v>355891510.08674401</v>
+        <v>3.0102067467839456e8</v>
       </c>
       <c r="F7">
-        <v>409396509.03496462</v>
+        <v>2.7909631850528204e8</v>
       </c>
       <c r="G7">
-        <v>351123650.51789606</v>
+        <v>2.563633141406557e8</v>
       </c>
       <c r="H7">
-        <v>367284396.57280999</v>
+        <v>4.353656611371059e8</v>
       </c>
       <c r="I7">
-        <v>240916564.79568711</v>
+        <v>4.874193358688112e8</v>
       </c>
       <c r="J7">
-        <v>305944424.76470387</v>
+        <v>3.2643216906794983e8</v>
       </c>
       <c r="K7">
-        <v>551925989.68367708</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3.786441164695561e8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
       <c r="A8" t="s">
         <v>17</v>
       </c>
       <c r="B8">
-        <v>179750708.71833512</v>
+        <v>1.8222790836330774e8</v>
       </c>
       <c r="C8">
-        <v>177383576.7628307</v>
+        <v>1.364619435127144e8</v>
       </c>
       <c r="D8">
-        <v>260540987.13047528</v>
+        <v>3.0009748542524177e8</v>
       </c>
       <c r="E8">
-        <v>335459535.01036924</v>
+        <v>3.5082085863620305e8</v>
       </c>
       <c r="F8">
-        <v>435108583.84398091</v>
+        <v>2.8407397550642216e8</v>
       </c>
       <c r="G8">
-        <v>372219184.51445502</v>
+        <v>4.980703501677943e8</v>
       </c>
       <c r="H8">
-        <v>152626433.71082819</v>
+        <v>2.359851364904509e7</v>
       </c>
       <c r="I8">
-        <v>662499468.14227664</v>
+        <v>9.681729448530605e8</v>
       </c>
       <c r="J8">
-        <v>748735595.61141121</v>
+        <v>8.698195964397902e8</v>
       </c>
       <c r="K8">
-        <v>1495074334.663096</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+        <v>8.14356763463235e8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
       <c r="A9" t="s">
         <v>18</v>
       </c>
       <c r="B9">
-        <v>590312479.82222867</v>
+        <v>6.490035230032277e8</v>
       </c>
       <c r="C9">
-        <v>716620045.95651305</v>
+        <v>6.874794482624598e8</v>
       </c>
       <c r="D9">
-        <v>737290919.57785952</v>
+        <v>7.954997233029366e8</v>
       </c>
       <c r="E9">
-        <v>584874938.61879194</v>
+        <v>7.234570633922147e8</v>
       </c>
       <c r="F9">
-        <v>714873878.19104528</v>
+        <v>9.527038929994347e8</v>
       </c>
       <c r="G9">
-        <v>788131268.64981842</v>
+        <v>7.580294737342256e8</v>
       </c>
       <c r="H9">
-        <v>851157200.2536819</v>
+        <v>9.043176412605233e8</v>
       </c>
       <c r="I9">
-        <v>776656029.75097919</v>
+        <v>9.330818483564837e8</v>
       </c>
       <c r="J9">
-        <v>875457329.12202775</v>
+        <v>9.570720637481767e8</v>
       </c>
       <c r="K9">
-        <v>1359865264.464958</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+        <v>9.309514971766104e8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
       <c r="A10" t="s">
         <v>19</v>
       </c>
       <c r="B10">
-        <v>682176582.40057123</v>
+        <v>5.859058196207265e8</v>
       </c>
       <c r="C10">
-        <v>645043251.14215493</v>
+        <v>6.492733873444312e8</v>
       </c>
       <c r="D10">
-        <v>676758831.59141445</v>
+        <v>4.728451598765224e8</v>
       </c>
       <c r="E10">
-        <v>990548518.8002466</v>
+        <v>8.990386225486628e8</v>
       </c>
       <c r="F10">
-        <v>904669292.31170619</v>
+        <v>7.590602151518909e8</v>
       </c>
       <c r="G10">
-        <v>806674818.32441175</v>
+        <v>1.1071024430642517e9</v>
       </c>
       <c r="H10">
-        <v>810369360.19954157</v>
+        <v>9.605560973767252e8</v>
       </c>
       <c r="I10">
-        <v>1718153652.1737084</v>
+        <v>3.017896697819526e8</v>
       </c>
       <c r="J10">
-        <v>1421470501.9782383</v>
+        <v>2.7334388817253456e9</v>
       </c>
       <c r="K10">
-        <v>2169610400.3336148</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+        <v>9.100161211157728e8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
       <c r="A11" t="s">
         <v>20</v>
       </c>
       <c r="B11">
-        <v>380593518.04141665</v>
+        <v>4.4796974978548884e8</v>
       </c>
       <c r="C11">
-        <v>357919789.86637127</v>
+        <v>3.5570733865049404e8</v>
       </c>
       <c r="D11">
-        <v>435511354.96055657</v>
+        <v>4.908236468663394e8</v>
       </c>
       <c r="E11">
-        <v>487193629.84509712</v>
+        <v>2.9066990928730905e8</v>
       </c>
       <c r="F11">
-        <v>346218455.28645641</v>
+        <v>3.2476585632757115e8</v>
       </c>
       <c r="G11">
-        <v>423784691.80780345</v>
+        <v>2.8928078041741127e8</v>
       </c>
       <c r="H11">
-        <v>687160358.78162241</v>
+        <v>4.764389558209741e8</v>
       </c>
       <c r="I11">
-        <v>123796046.04026081</v>
+        <v>4.428160773147188e8</v>
       </c>
       <c r="J11">
-        <v>631134833.0587765</v>
+        <v>5.778417993951914e8</v>
       </c>
       <c r="K11">
-        <v>178203466.81670186</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3.214017235980747e8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
       <c r="A12" t="s">
         <v>21</v>
       </c>
       <c r="B12">
-        <v>610459483.7845149</v>
+        <v>7.029523830224525e8</v>
       </c>
       <c r="C12">
-        <v>662382417.78929472</v>
+        <v>5.870053192368141e8</v>
       </c>
       <c r="D12">
-        <v>707221998.80727971</v>
+        <v>6.547204856796716e8</v>
       </c>
       <c r="E12">
-        <v>719538038.46970618</v>
+        <v>6.790660228736749e8</v>
       </c>
       <c r="F12">
-        <v>643903750.36717081</v>
+        <v>6.094447748790439e8</v>
       </c>
       <c r="G12">
-        <v>520213141.28565228</v>
+        <v>5.542851444455905e8</v>
       </c>
       <c r="H12">
-        <v>646467265.35945833</v>
+        <v>8.417519723276896e8</v>
       </c>
       <c r="I12">
-        <v>487334457.95618826</v>
+        <v>8.844673542245121e8</v>
       </c>
       <c r="J12">
-        <v>541187785.14317989</v>
+        <v>6.750774097282137e8</v>
       </c>
       <c r="K12">
-        <v>997154580.44498408</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+        <v>7.348517545098993e8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
       <c r="A13" t="s">
         <v>22</v>
       </c>
       <c r="B13">
-        <v>444694978.87685806</v>
+        <v>3.33343025565202e8</v>
       </c>
       <c r="C13">
-        <v>326062352.70833385</v>
+        <v>3.4698455808060974e8</v>
       </c>
       <c r="D13">
-        <v>457442151.07946384</v>
+        <v>4.0037944216314846e8</v>
       </c>
       <c r="E13">
-        <v>271621638.97737724</v>
+        <v>8.338458466526533e8</v>
       </c>
       <c r="F13">
-        <v>135936333.51880071</v>
+        <v>2.0653265145948195e8</v>
       </c>
       <c r="G13">
-        <v>700203630.08449709</v>
+        <v>6.375099997058067e8</v>
       </c>
       <c r="H13">
-        <v>463329751.63105333</v>
+        <v>3.117301316574522e8</v>
       </c>
       <c r="I13">
-        <v>330267378.23485839</v>
+        <v>8.328245762038274e8</v>
       </c>
       <c r="J13">
-        <v>749961148.83138394</v>
+        <v>6.0359105066415e8</v>
       </c>
       <c r="K13">
-        <v>786429751.87875938</v>
+        <v>1.3214958473890986e9</v>
       </c>
     </row>
   </sheetData>
@@ -921,11 +910,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7372E833-5FD7-42CF-9CB2-CCCFF1033FE9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF0E20E-E4D8-9B45-9C94-E89B574F109C}">
   <dimension ref="A1:K13"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -960,424 +949,424 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
         <v>11</v>
       </c>
       <c r="B2">
-        <v>234549687.32188326</v>
+        <v>2.3211087910909268e8</v>
       </c>
       <c r="C2">
-        <v>223928845.90141809</v>
+        <v>2.9848826589480096e8</v>
       </c>
       <c r="D2">
-        <v>241636034.53981224</v>
+        <v>2.3863081649476895e8</v>
       </c>
       <c r="E2">
-        <v>302873864.98625612</v>
+        <v>3.453493630371045e8</v>
       </c>
       <c r="F2">
-        <v>310830951.43569833</v>
+        <v>3.080929178623604e8</v>
       </c>
       <c r="G2">
-        <v>397435186.26740998</v>
+        <v>4.8362579803140026e8</v>
       </c>
       <c r="H2">
-        <v>294089393.15786213</v>
+        <v>2.2723266100013375e8</v>
       </c>
       <c r="I2">
-        <v>339904079.02949423</v>
+        <v>3.7049238871555966e8</v>
       </c>
       <c r="J2">
-        <v>468608590.46325952</v>
+        <v>6.15668303139034e8</v>
       </c>
       <c r="K2">
-        <v>369212768.24848801</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1.9242230978112292e8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3" t="s">
         <v>12</v>
       </c>
       <c r="B3">
-        <v>555020433.14300287</v>
+        <v>3.111773395116339e8</v>
       </c>
       <c r="C3">
-        <v>520547162.88335651</v>
+        <v>3.348218375828177e8</v>
       </c>
       <c r="D3">
-        <v>359375508.53346103</v>
+        <v>8.113416582579339e8</v>
       </c>
       <c r="E3">
-        <v>594062284.93677258</v>
+        <v>6.5699163764135e8</v>
       </c>
       <c r="F3">
-        <v>1056442057.7685559</v>
+        <v>9.071922406612762e8</v>
       </c>
       <c r="G3">
-        <v>591678857.96792793</v>
+        <v>6.891098391319757e8</v>
       </c>
       <c r="H3">
-        <v>727321232.66377282</v>
+        <v>1.325448866558319e9</v>
       </c>
       <c r="I3">
-        <v>1218659760.9773154</v>
+        <v>1.3574254213979917e9</v>
       </c>
       <c r="J3">
-        <v>1668179191.5095899</v>
+        <v>5.1409260594144136e8</v>
       </c>
       <c r="K3">
-        <v>188273538.71237421</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1.94351199092586e9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
       <c r="A4" t="s">
         <v>13</v>
       </c>
       <c r="B4">
-        <v>26807519.493087843</v>
+        <v>1.8357784575865522e7</v>
       </c>
       <c r="C4">
-        <v>20583374.694766823</v>
+        <v>2.08122496466083e7</v>
       </c>
       <c r="D4">
-        <v>30931176.905525409</v>
+        <v>1.4193943145557776e7</v>
       </c>
       <c r="E4">
-        <v>38731676.423083283</v>
+        <v>3.710009495224252e7</v>
       </c>
       <c r="F4">
-        <v>29009664.787545756</v>
+        <v>2.5125443239725925e7</v>
       </c>
       <c r="G4">
-        <v>32662040.305258632</v>
+        <v>3.853278470527064e7</v>
       </c>
       <c r="H4">
-        <v>61705479.09819252</v>
+        <v>5.950543202169565e7</v>
       </c>
       <c r="I4">
-        <v>91210738.992935389</v>
+        <v>4.023283552383763e7</v>
       </c>
       <c r="J4">
-        <v>30602773.135495987</v>
+        <v>9.082706326528552e7</v>
       </c>
       <c r="K4">
-        <v>129506209.81513061</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1.0520322498769993e8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
       <c r="A5" t="s">
         <v>14</v>
       </c>
       <c r="B5">
-        <v>27216530.880601194</v>
+        <v>2.848584478429758e7</v>
       </c>
       <c r="C5">
-        <v>36128820.363646343</v>
+        <v>3.696631784791036e7</v>
       </c>
       <c r="D5">
-        <v>40430621.108659327</v>
+        <v>4.20501613198183e7</v>
       </c>
       <c r="E5">
-        <v>50185652.376320072</v>
+        <v>4.391036972810015e7</v>
       </c>
       <c r="F5">
-        <v>58990672.832436979</v>
+        <v>5.4048566791496396e7</v>
       </c>
       <c r="G5">
-        <v>57842494.695028007</v>
+        <v>5.778858036313352e7</v>
       </c>
       <c r="H5">
-        <v>64390332.846368425</v>
+        <v>7.388879896104623e7</v>
       </c>
       <c r="I5">
-        <v>68797373.021729708</v>
+        <v>7.896752547374727e7</v>
       </c>
       <c r="J5">
-        <v>71299092.040560693</v>
+        <v>7.726531048375529e7</v>
       </c>
       <c r="K5">
-        <v>90851011.587240875</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+        <v>8.065546617272887e7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
       <c r="A6" t="s">
         <v>15</v>
       </c>
       <c r="B6">
-        <v>303995732.77633232</v>
+        <v>3.1183934574209976e8</v>
       </c>
       <c r="C6">
-        <v>319382223.82155424</v>
+        <v>3.6144812246308887e8</v>
       </c>
       <c r="D6">
-        <v>335378074.29451716</v>
+        <v>3.324308447619791e8</v>
       </c>
       <c r="E6">
-        <v>386112572.7099039</v>
+        <v>3.8382665230767584e8</v>
       </c>
       <c r="F6">
-        <v>316427330.43293452</v>
+        <v>4.0210361341776705e8</v>
       </c>
       <c r="G6">
-        <v>333769944.1010679</v>
+        <v>3.637629279364848e8</v>
       </c>
       <c r="H6">
-        <v>408308807.9245553</v>
+        <v>3.647303173693133e8</v>
       </c>
       <c r="I6">
-        <v>349337166.73017466</v>
+        <v>4.008994188748239e8</v>
       </c>
       <c r="J6">
-        <v>466206244.33542776</v>
+        <v>3.7946342814196825e8</v>
       </c>
       <c r="K6">
-        <v>411142327.38671285</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+        <v>4.755488963312707e8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
       <c r="A7" t="s">
         <v>16</v>
       </c>
       <c r="B7">
-        <v>338485449.21751916</v>
+        <v>3.749244860753849e8</v>
       </c>
       <c r="C7">
-        <v>297220409.07591468</v>
+        <v>3.522869909055479e8</v>
       </c>
       <c r="D7">
-        <v>366683469.37284839</v>
+        <v>3.795526193737042e8</v>
       </c>
       <c r="E7">
-        <v>347955285.61961508</v>
+        <v>4.1159540724359715e8</v>
       </c>
       <c r="F7">
-        <v>430318446.06129318</v>
+        <v>2.649443906953663e8</v>
       </c>
       <c r="G7">
-        <v>318458768.60102296</v>
+        <v>3.319994992170885e8</v>
       </c>
       <c r="H7">
-        <v>384751655.40185624</v>
+        <v>3.8620144828387386e8</v>
       </c>
       <c r="I7">
-        <v>408000848.37349391</v>
+        <v>3.9185078596209013e8</v>
       </c>
       <c r="J7">
-        <v>391897839.42408711</v>
+        <v>3.911272287612296e8</v>
       </c>
       <c r="K7">
-        <v>448603704.32690382</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+        <v>2.271130827958227e8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
       <c r="A8" t="s">
         <v>17</v>
       </c>
       <c r="B8">
-        <v>177734931.85308132</v>
+        <v>2.0769384469078794e8</v>
       </c>
       <c r="C8">
-        <v>226265420.48745552</v>
+        <v>1.5799646966925994e8</v>
       </c>
       <c r="D8">
-        <v>263132776.34329641</v>
+        <v>2.8674028342440295e8</v>
       </c>
       <c r="E8">
-        <v>445182342.85567749</v>
+        <v>2.115447831351004e8</v>
       </c>
       <c r="F8">
-        <v>390402037.92083007</v>
+        <v>2.0839409198570365e8</v>
       </c>
       <c r="G8">
-        <v>550272159.9821713</v>
+        <v>3.3476833372704965e8</v>
       </c>
       <c r="H8">
-        <v>263016041.81828746</v>
+        <v>1.778587548726809e8</v>
       </c>
       <c r="I8">
-        <v>683589610.37428248</v>
+        <v>8.606470197317667e8</v>
       </c>
       <c r="J8">
-        <v>348911804.62992543</v>
+        <v>7.867729108073854e8</v>
       </c>
       <c r="K8">
-        <v>415599274.74684316</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+        <v>7.077212493485593e8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
       <c r="A9" t="s">
         <v>18</v>
       </c>
       <c r="B9">
-        <v>681356906.58583272</v>
+        <v>5.657696024704907e8</v>
       </c>
       <c r="C9">
-        <v>623545721.43767846</v>
+        <v>6.902722991834769e8</v>
       </c>
       <c r="D9">
-        <v>776804896.8511548</v>
+        <v>7.940044997059581e8</v>
       </c>
       <c r="E9">
-        <v>672533585.73929989</v>
+        <v>6.427951095657427e8</v>
       </c>
       <c r="F9">
-        <v>955052555.61860716</v>
+        <v>8.799273445287563e8</v>
       </c>
       <c r="G9">
-        <v>696308185.10701621</v>
+        <v>8.69955168463791e8</v>
       </c>
       <c r="H9">
-        <v>636040505.42461681</v>
+        <v>7.83465257707859e8</v>
       </c>
       <c r="I9">
-        <v>684840408.05936646</v>
+        <v>1.140714618733327e9</v>
       </c>
       <c r="J9">
-        <v>921767425.51295042</v>
+        <v>9.847533674185572e8</v>
       </c>
       <c r="K9">
-        <v>618311700.89919114</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+        <v>1.2350933143509128e9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
       <c r="A10" t="s">
         <v>19</v>
       </c>
       <c r="B10">
-        <v>646255361.24162734</v>
+        <v>7.14643883025544e8</v>
       </c>
       <c r="C10">
-        <v>697729808.113392</v>
+        <v>7.583556734605304e8</v>
       </c>
       <c r="D10">
-        <v>853654000.58250415</v>
+        <v>9.556471472101068e8</v>
       </c>
       <c r="E10">
-        <v>834540616.24723971</v>
+        <v>6.459394980499601e8</v>
       </c>
       <c r="F10">
-        <v>1142296730.1325696</v>
+        <v>1.27118217826647e9</v>
       </c>
       <c r="G10">
-        <v>825097360.36621761</v>
+        <v>1.2130544406386492e9</v>
       </c>
       <c r="H10">
-        <v>1490104965.5807939</v>
+        <v>1.1421993855304036e9</v>
       </c>
       <c r="I10">
-        <v>1137992866.4229038</v>
+        <v>1.8840876026023438e9</v>
       </c>
       <c r="J10">
-        <v>2520102508.1367903</v>
+        <v>2.594110822230082e9</v>
       </c>
       <c r="K10">
-        <v>3538519113.1622062</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+        <v>3.0315496024717636e9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
       <c r="A11" t="s">
         <v>20</v>
       </c>
       <c r="B11">
-        <v>432754523.62804711</v>
+        <v>4.3033884276909167e8</v>
       </c>
       <c r="C11">
-        <v>493342708.56246436</v>
+        <v>3.009902913041657e8</v>
       </c>
       <c r="D11">
-        <v>279629060.94752836</v>
+        <v>4.47213365434397e8</v>
       </c>
       <c r="E11">
-        <v>397188085.02526605</v>
+        <v>2.9429474773458135e8</v>
       </c>
       <c r="F11">
-        <v>234658590.65599421</v>
+        <v>5.402335242866758e8</v>
       </c>
       <c r="G11">
-        <v>383805332.0615769</v>
+        <v>4.14789199301885e8</v>
       </c>
       <c r="H11">
-        <v>416771168.26363051</v>
+        <v>5.33524315542758e8</v>
       </c>
       <c r="I11">
-        <v>462817362.13680798</v>
+        <v>5.817523091625973e8</v>
       </c>
       <c r="J11">
-        <v>637480132.80154824</v>
+        <v>4.588481771240103e8</v>
       </c>
       <c r="K11">
-        <v>316085762.2810868</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+        <v>6.086724940632217e8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
       <c r="A12" t="s">
         <v>21</v>
       </c>
       <c r="B12">
-        <v>611186226.38604701</v>
+        <v>5.706050739175953e8</v>
       </c>
       <c r="C12">
-        <v>610638159.21117377</v>
+        <v>6.222136972111194e8</v>
       </c>
       <c r="D12">
-        <v>683458152.72743273</v>
+        <v>6.999760386218611e8</v>
       </c>
       <c r="E12">
-        <v>634855966.61096895</v>
+        <v>8.001180843998573e8</v>
       </c>
       <c r="F12">
-        <v>676884008.38035989</v>
+        <v>6.616634611605746e8</v>
       </c>
       <c r="G12">
-        <v>545814956.22321343</v>
+        <v>7.14238595223895e8</v>
       </c>
       <c r="H12">
-        <v>832811682.13957179</v>
+        <v>7.610427313978678e8</v>
       </c>
       <c r="I12">
-        <v>613992476.73472786</v>
+        <v>5.902776620027502e8</v>
       </c>
       <c r="J12">
-        <v>673745147.20365524</v>
+        <v>7.825983329825139e8</v>
       </c>
       <c r="K12">
-        <v>685423202.27466333</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+        <v>6.81799766813164e8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
       <c r="A13" t="s">
         <v>22</v>
       </c>
       <c r="B13">
-        <v>560668762.91228616</v>
+        <v>3.764750026255865e8</v>
       </c>
       <c r="C13">
-        <v>305286970.67246145</v>
+        <v>5.585462431161689e8</v>
       </c>
       <c r="D13">
-        <v>264344757.11120865</v>
+        <v>6.776617400621051e8</v>
       </c>
       <c r="E13">
-        <v>325837660.49708134</v>
+        <v>2.920174116715634e8</v>
       </c>
       <c r="F13">
-        <v>458145145.1251334</v>
+        <v>4.692527143034406e8</v>
       </c>
       <c r="G13">
-        <v>529777321.37764257</v>
+        <v>7.770676517117692e8</v>
       </c>
       <c r="H13">
-        <v>574831262.86825943</v>
+        <v>5.1870733314573973e8</v>
       </c>
       <c r="I13">
-        <v>846037425.70948875</v>
+        <v>1.178546701636892e8</v>
       </c>
       <c r="J13">
-        <v>503930011.20133662</v>
+        <v>1.3058848795772977e9</v>
       </c>
       <c r="K13">
-        <v>307078175.46628827</v>
+        <v>7.351009707740635e8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>